<commit_message>
update 2. took the rat out
</commit_message>
<xml_diff>
--- a/assets/AssetDB.xlsx
+++ b/assets/AssetDB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TEMP\Crawler-Projektpraktikum\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8B6C4A-CE51-4448-BD6B-FBC5F2DCB6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2DDC4F1-2695-4E94-AF8E-A98F1BE39359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{B3F5CE5B-25EC-484D-8705-D10708A494B7}"/>
   </bookViews>
@@ -40,7 +40,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="113">
+  <futureMetadata name="XLRICHVALUE" count="112">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -825,15 +825,8 @@
         </ext>
       </extLst>
     </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="112"/>
-        </ext>
-      </extLst>
-    </bk>
   </futureMetadata>
-  <valueMetadata count="113">
+  <valueMetadata count="112">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -1169,16 +1162,13 @@
     </bk>
     <bk>
       <rc t="1" v="111"/>
-    </bk>
-    <bk>
-      <rc t="1" v="112"/>
     </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="166">
   <si>
     <t>Category</t>
   </si>
@@ -1271,15 +1261,6 @@
   </si>
   <si>
     <t>Player Character</t>
-  </si>
-  <si>
-    <t>rat.png</t>
-  </si>
-  <si>
-    <t>NPCs</t>
-  </si>
-  <si>
-    <t>???</t>
   </si>
   <si>
     <t>rat-merchant-rug.png</t>
@@ -2270,13 +2251,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1</xdr:colOff>
-      <xdr:row>88</xdr:row>
+      <xdr:row>87</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1048167</xdr:colOff>
-      <xdr:row>89</xdr:row>
+      <xdr:colOff>1044357</xdr:colOff>
+      <xdr:row>88</xdr:row>
       <xdr:rowOff>1474</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2331,13 +2312,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>89</xdr:row>
+      <xdr:row>88</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>90</xdr:row>
+      <xdr:row>89</xdr:row>
       <xdr:rowOff>1115</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2392,14 +2373,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>90</xdr:row>
+      <xdr:row>89</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>15624</xdr:colOff>
-      <xdr:row>91</xdr:row>
-      <xdr:rowOff>2662</xdr:rowOff>
+      <xdr:colOff>19434</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>2661</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2453,14 +2434,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1</xdr:colOff>
-      <xdr:row>91</xdr:row>
+      <xdr:row>90</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>15458</xdr:colOff>
-      <xdr:row>92</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
+      <xdr:colOff>19268</xdr:colOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>2</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2514,13 +2495,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>2</xdr:colOff>
-      <xdr:row>92</xdr:row>
+      <xdr:row>91</xdr:row>
       <xdr:rowOff>9909</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>16393</xdr:colOff>
-      <xdr:row>92</xdr:row>
+      <xdr:colOff>20203</xdr:colOff>
+      <xdr:row>91</xdr:row>
       <xdr:rowOff>727238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2615,7 +2596,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="113">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="112">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -3062,10 +3043,6 @@
   </rv>
   <rv s="0">
     <v>111</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>112</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -3194,13 +3171,12 @@
   <rel r:id="rId110"/>
   <rel r:id="rId111"/>
   <rel r:id="rId112"/>
-  <rel r:id="rId113"/>
 </richValueRels>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33703373-9280-482F-8933-8BD3E9BA98E3}" name="Table1" displayName="Table1" ref="A1:D52" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4">
-  <autoFilter ref="A1:D52" xr:uid="{33703373-9280-482F-8933-8BD3E9BA98E3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33703373-9280-482F-8933-8BD3E9BA98E3}" name="Table1" displayName="Table1" ref="A1:D51" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4">
+  <autoFilter ref="A1:D51" xr:uid="{33703373-9280-482F-8933-8BD3E9BA98E3}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{E1B98A4C-EE91-454F-B8D7-8CF3EEAB7D54}" name="Category" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{1FDB1714-61BC-4DE3-9510-5783E3C5F52E}" name="Name" dataDxfId="2"/>
@@ -3528,7 +3504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D18B40B6-A108-4343-8456-7741D8A067D3}">
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:D122"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
@@ -3616,7 +3592,7 @@
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3630,7 +3606,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3644,7 +3620,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -3658,7 +3634,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -3672,7 +3648,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3806,13 +3782,13 @@
         <v>30</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C20" s="17" t="e" vm="18">
         <v>#VALUE!</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3820,41 +3796,41 @@
         <v>30</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C21" s="17" t="e" vm="19">
         <v>#VALUE!</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="13" t="e" vm="20">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="2" t="e" vm="20">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" s="12" t="s">
+      <c r="C23" s="2" t="e" vm="21">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>34</v>
-      </c>
-      <c r="C23" s="13" t="e" vm="21">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -3862,195 +3838,195 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C24" s="2" t="e" vm="22">
         <v>#VALUE!</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="2" t="e" vm="23">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>36</v>
-      </c>
-      <c r="C25" s="2" t="e" vm="23">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" s="2" t="e" vm="24">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="2" t="e" vm="24">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D26" s="9" t="s">
+      <c r="C27" s="13" t="e" vm="25">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="8" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B27" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="2" t="e" vm="25">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="13" t="e" vm="26">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>39</v>
+      <c r="C28" s="2" t="e" vm="26">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C29" s="2" t="e" vm="27">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="C30" s="2" t="e" vm="28">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C29" s="2" t="e" vm="27">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D29" s="9" t="s">
+      <c r="C31" s="2" t="e" vm="29">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
+      <c r="B32" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C32" s="13" t="e" vm="30">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C30" s="2" t="e" vm="28">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="8" t="s">
+      <c r="B33" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" s="2" t="e" vm="31">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C31" s="2" t="e" vm="29">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C32" s="2" t="e" vm="30">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="C33" s="13" t="e" vm="31">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
-        <v>19</v>
-      </c>
       <c r="B34" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C34" s="2" t="e" vm="32">
         <v>#VALUE!</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D34" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>9</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C35" s="2" t="e" vm="33">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C36" s="13" t="e" vm="34">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D36" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C35" s="2" t="e" vm="33">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C36" s="2" t="e" vm="34">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C37" s="13" t="e" vm="35">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D37" s="10" t="s">
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>55</v>
+      </c>
+      <c r="C37" s="2" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
@@ -4058,410 +4034,410 @@
         <v>19</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C38" s="2" t="e" vm="36">
         <v>#VALUE!</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" s="2" t="e" vm="37">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C39" s="2" t="e" vm="37">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="8" t="s">
+      <c r="B40" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="C40" s="2" t="e" vm="38">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C40" s="2" t="e" vm="38">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="8" t="s">
+      <c r="B41" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="C41" s="2" t="e" vm="39">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D41" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C41" s="2" t="e" vm="39">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="8" t="s">
+      <c r="A42" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B42" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C42" s="2" t="e" vm="40">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D42" s="22" t="s">
-        <v>66</v>
+      <c r="C42" s="13" t="e" vm="40">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C43" s="13" t="e" vm="41">
         <v>#VALUE!</v>
       </c>
-      <c r="D43" s="14" t="s">
-        <v>66</v>
+      <c r="D43" s="21" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B44" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C44" s="13" t="e" vm="42">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D44" s="21" t="s">
         <v>69</v>
-      </c>
-      <c r="C44" s="13" t="e" vm="42">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D44" s="21" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B45" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="C45" s="13" t="e" vm="43">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D45" s="21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="C45" s="13" t="e" vm="43">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D45" s="21" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="11" t="s">
-        <v>68</v>
-      </c>
       <c r="B46" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C46" s="13" t="e" vm="44">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D46" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
+      </c>
+      <c r="C46" s="2" t="e" vm="44">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D46" s="23" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B47" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B47" s="12" t="s">
-        <v>77</v>
-      </c>
       <c r="C47" s="2" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="C48" s="2" t="e" vm="46">
+        <v>72</v>
+      </c>
+      <c r="C48" s="13" t="e" vm="46">
         <v>#VALUE!</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B49" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C49" s="2" t="e" vm="47">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D49" s="23" t="s">
         <v>75</v>
-      </c>
-      <c r="C49" s="13" t="e" vm="47">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D49" s="23" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C50" s="2" t="e" vm="48">
         <v>#VALUE!</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="C51" s="2" t="e" vm="49">
+        <v>78</v>
+      </c>
+      <c r="C51" s="13" t="e" vm="49">
         <v>#VALUE!</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A52" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="C52" s="13" t="e" vm="50">
+        <v>79</v>
+      </c>
+      <c r="C52" s="2" t="e" vm="50">
         <v>#VALUE!</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A53" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B53" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C53" s="2" t="e" vm="51">
         <v>#VALUE!</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C54" s="2" t="e" vm="52">
+        <v>81</v>
+      </c>
+      <c r="C54" s="13" t="e" vm="52">
         <v>#VALUE!</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A55" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B55" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="C55" s="13" t="e" vm="53">
+        <v>82</v>
+      </c>
+      <c r="C55" s="2" t="e" vm="53">
         <v>#VALUE!</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C56" s="2" t="e" vm="54">
         <v>#VALUE!</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B57" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C57" s="13" t="e" vm="55">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D57" s="23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="C57" s="2" t="e" vm="55">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D57" s="23" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A58" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="B58" s="12" t="s">
+      <c r="C58" t="e" vm="56">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D58" s="27" t="s">
         <v>87</v>
-      </c>
-      <c r="C58" s="13" t="e" vm="56">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D58" s="23" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B59" s="25" t="s">
-        <v>89</v>
-      </c>
       <c r="C59" t="e" vm="57">
         <v>#VALUE!</v>
       </c>
       <c r="D59" s="27" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B60" s="25" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C60" t="e" vm="58">
         <v>#VALUE!</v>
       </c>
       <c r="D60" s="27" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A61" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B61" s="25" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="B61" s="25" t="s">
-        <v>92</v>
-      </c>
       <c r="C61" t="e" vm="59">
         <v>#VALUE!</v>
       </c>
       <c r="D61" s="27" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B62" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="C62" t="e" vm="60">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D62" s="27" t="s">
         <v>93</v>
-      </c>
-      <c r="C62" t="e" vm="60">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D62" s="27" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A63" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B63" s="25" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C63" t="e" vm="61">
         <v>#VALUE!</v>
       </c>
       <c r="D63" s="27" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B64" s="25" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C64" t="e" vm="62">
         <v>#VALUE!</v>
       </c>
       <c r="D64" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A65" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B65" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="C65" t="e" vm="63">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D65" s="27" t="s">
         <v>97</v>
-      </c>
-      <c r="C65" t="e" vm="63">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D65" s="27" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B66" s="25" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C66" t="e" vm="64">
         <v>#VALUE!</v>
       </c>
       <c r="D66" s="27" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B67" s="25" t="s">
         <v>99</v>
@@ -4470,301 +4446,298 @@
         <v>#VALUE!</v>
       </c>
       <c r="D67" s="27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B68" s="25" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C68" t="e" vm="66">
         <v>#VALUE!</v>
       </c>
       <c r="D68" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B69" s="25" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C69" t="e" vm="67">
         <v>#VALUE!</v>
       </c>
       <c r="D69" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B70" s="25" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C70" t="e" vm="68">
         <v>#VALUE!</v>
       </c>
       <c r="D70" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B71" s="25" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C71" t="e" vm="69">
         <v>#VALUE!</v>
       </c>
       <c r="D71" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B72" s="25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C72" t="e" vm="70">
         <v>#VALUE!</v>
       </c>
       <c r="D72" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B73" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C73" t="e" vm="71">
         <v>#VALUE!</v>
       </c>
       <c r="D73" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B74" s="25" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C74" t="e" vm="72">
         <v>#VALUE!</v>
       </c>
       <c r="D74" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B75" s="25" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C75" t="e" vm="73">
         <v>#VALUE!</v>
       </c>
       <c r="D75" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B76" s="25" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C76" t="e" vm="74">
         <v>#VALUE!</v>
       </c>
       <c r="D76" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B77" s="25" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C77" t="e" vm="75">
         <v>#VALUE!</v>
       </c>
       <c r="D77" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B78" s="25" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C78" t="e" vm="76">
         <v>#VALUE!</v>
       </c>
       <c r="D78" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B79" s="25" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C79" t="e" vm="77">
         <v>#VALUE!</v>
       </c>
       <c r="D79" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B80" s="25" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C80" t="e" vm="78">
         <v>#VALUE!</v>
       </c>
       <c r="D80" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B81" s="25" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C81" t="e" vm="79">
         <v>#VALUE!</v>
       </c>
       <c r="D81" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B82" s="25" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C82" t="e" vm="80">
         <v>#VALUE!</v>
       </c>
       <c r="D82" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B83" s="25" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C83" t="e" vm="81">
         <v>#VALUE!</v>
       </c>
       <c r="D83" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="24" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B84" s="25" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C84" t="e" vm="82">
         <v>#VALUE!</v>
       </c>
       <c r="D84" s="27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="B85" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="B85" t="s">
+        <v>118</v>
+      </c>
+      <c r="C85" t="e" vm="83">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D85" t="s">
         <v>119</v>
-      </c>
-      <c r="C85" t="e" vm="83">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D85" s="27" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="28" t="s">
         <v>121</v>
       </c>
       <c r="C86" t="e" vm="84">
         <v>#VALUE!</v>
       </c>
       <c r="D86" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A87" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B87" s="28" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" s="24" t="s">
+      <c r="C87" t="e" vm="85">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D87" s="29" t="s">
         <v>123</v>
       </c>
-      <c r="B87" s="28" t="s">
-        <v>124</v>
-      </c>
-      <c r="C87" t="e" vm="85">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D87" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="88" spans="1:4" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B88" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="D88" s="29" t="s">
         <v>125</v>
-      </c>
-      <c r="C88" t="e" vm="86">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D88" s="29" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -4772,10 +4745,10 @@
         <v>19</v>
       </c>
       <c r="B89" s="28" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D89" s="29" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -4783,10 +4756,10 @@
         <v>19</v>
       </c>
       <c r="B90" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="D90" s="29" t="s">
         <v>127</v>
-      </c>
-      <c r="D90" s="29" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -4794,74 +4767,77 @@
         <v>19</v>
       </c>
       <c r="B91" s="28" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D91" s="29" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D92" s="29" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B93" s="28" t="s">
-        <v>127</v>
-      </c>
-      <c r="D93" s="29" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B93" t="s">
+        <v>157</v>
+      </c>
+      <c r="C93" t="e" vm="86">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D93" s="26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="87" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B94" t="s">
+        <v>156</v>
+      </c>
+      <c r="C94" t="e" vm="87">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D94" t="s">
         <v>160</v>
       </c>
-      <c r="C94" t="e" vm="87">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D94" s="26" t="s">
+    </row>
+    <row r="95" spans="1:4" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="B95" t="s">
+        <v>155</v>
+      </c>
+      <c r="C95" t="e" vm="88">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D95" s="26" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="95" spans="1:4" ht="87" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="24" t="s">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B95" t="s">
-        <v>159</v>
-      </c>
-      <c r="C95" t="e" vm="88">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D95" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="24" t="s">
-        <v>133</v>
-      </c>
       <c r="B96" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="C96" t="e" vm="89">
         <v>#VALUE!</v>
       </c>
-      <c r="D96" s="26" t="s">
-        <v>166</v>
+      <c r="D96" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
@@ -4869,13 +4845,13 @@
         <v>19</v>
       </c>
       <c r="B97" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C97" t="e" vm="90">
         <v>#VALUE!</v>
       </c>
       <c r="D97" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
@@ -4883,13 +4859,13 @@
         <v>19</v>
       </c>
       <c r="B98" t="s">
-        <v>141</v>
-      </c>
-      <c r="C98" t="e" vm="91">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D98" t="s">
-        <v>165</v>
+        <v>133</v>
+      </c>
+      <c r="C98" t="e" vm="17">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D98" s="26" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
@@ -4897,13 +4873,13 @@
         <v>19</v>
       </c>
       <c r="B99" t="s">
-        <v>136</v>
-      </c>
-      <c r="C99" t="e" vm="17">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D99" s="26" t="s">
-        <v>20</v>
+        <v>134</v>
+      </c>
+      <c r="C99" t="e" vm="91">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D99" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
@@ -4911,41 +4887,41 @@
         <v>19</v>
       </c>
       <c r="B100" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C100" t="e" vm="92">
         <v>#VALUE!</v>
       </c>
       <c r="D100" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B101" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C101" t="e" vm="93">
         <v>#VALUE!</v>
       </c>
       <c r="D101" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B102" t="s">
-        <v>139</v>
+        <v>38</v>
       </c>
       <c r="C102" t="e" vm="94">
         <v>#VALUE!</v>
       </c>
       <c r="D102" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
@@ -4953,13 +4929,13 @@
         <v>19</v>
       </c>
       <c r="B103" t="s">
-        <v>41</v>
+        <v>139</v>
       </c>
       <c r="C103" t="e" vm="95">
         <v>#VALUE!</v>
       </c>
       <c r="D103" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
@@ -4967,55 +4943,55 @@
         <v>19</v>
       </c>
       <c r="B104" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C104" t="e" vm="96">
         <v>#VALUE!</v>
       </c>
       <c r="D104" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B105" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="C105" t="e" vm="97">
         <v>#VALUE!</v>
       </c>
       <c r="D105" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B106" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C106" t="e" vm="98">
         <v>#VALUE!</v>
       </c>
       <c r="D106" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B107" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C107" t="e" vm="99">
         <v>#VALUE!</v>
       </c>
       <c r="D107" t="s">
-        <v>168</v>
+        <v>63</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
@@ -5023,13 +4999,13 @@
         <v>19</v>
       </c>
       <c r="B108" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C108" t="e" vm="100">
         <v>#VALUE!</v>
       </c>
       <c r="D108" t="s">
-        <v>66</v>
+        <v>20</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
@@ -5037,9 +5013,9 @@
         <v>19</v>
       </c>
       <c r="B109" t="s">
-        <v>154</v>
-      </c>
-      <c r="C109" t="e" vm="101">
+        <v>27</v>
+      </c>
+      <c r="C109" t="e" vm="15">
         <v>#VALUE!</v>
       </c>
       <c r="D109" t="s">
@@ -5051,9 +5027,9 @@
         <v>19</v>
       </c>
       <c r="B110" t="s">
-        <v>27</v>
-      </c>
-      <c r="C110" t="e" vm="15">
+        <v>150</v>
+      </c>
+      <c r="C110" t="e" vm="101">
         <v>#VALUE!</v>
       </c>
       <c r="D110" t="s">
@@ -5065,7 +5041,7 @@
         <v>19</v>
       </c>
       <c r="B111" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C111" t="e" vm="102">
         <v>#VALUE!</v>
@@ -5079,7 +5055,7 @@
         <v>19</v>
       </c>
       <c r="B112" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C112" t="e" vm="103">
         <v>#VALUE!</v>
@@ -5093,7 +5069,7 @@
         <v>19</v>
       </c>
       <c r="B113" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C113" t="e" vm="104">
         <v>#VALUE!</v>
@@ -5107,13 +5083,13 @@
         <v>19</v>
       </c>
       <c r="B114" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C114" t="e" vm="105">
         <v>#VALUE!</v>
       </c>
       <c r="D114" t="s">
-        <v>20</v>
+        <v>131</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
@@ -5121,13 +5097,13 @@
         <v>19</v>
       </c>
       <c r="B115" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C115" t="e" vm="106">
         <v>#VALUE!</v>
       </c>
       <c r="D115" t="s">
-        <v>134</v>
+        <v>20</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
@@ -5135,7 +5111,7 @@
         <v>19</v>
       </c>
       <c r="B116" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C116" t="e" vm="107">
         <v>#VALUE!</v>
@@ -5149,7 +5125,7 @@
         <v>19</v>
       </c>
       <c r="B117" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C117" t="e" vm="108">
         <v>#VALUE!</v>
@@ -5163,7 +5139,7 @@
         <v>19</v>
       </c>
       <c r="B118" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C118" t="e" vm="109">
         <v>#VALUE!</v>
@@ -5177,7 +5153,7 @@
         <v>19</v>
       </c>
       <c r="B119" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="C119" t="e" vm="110">
         <v>#VALUE!</v>
@@ -5186,12 +5162,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="24" t="s">
-        <v>19</v>
+        <v>130</v>
       </c>
       <c r="B120" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C120" t="e" vm="111">
         <v>#VALUE!</v>
@@ -5200,46 +5176,32 @@
         <v>20</v>
       </c>
     </row>
-    <row r="121" spans="1:4" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" s="24" t="s">
-        <v>133</v>
+        <v>19</v>
       </c>
       <c r="B121" t="s">
-        <v>144</v>
-      </c>
-      <c r="C121" t="e" vm="112">
+        <v>26</v>
+      </c>
+      <c r="C121" t="e" vm="14">
         <v>#VALUE!</v>
       </c>
       <c r="D121" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B122" t="s">
-        <v>26</v>
-      </c>
-      <c r="C122" t="e" vm="14">
+        <v>158</v>
+      </c>
+      <c r="C122" t="e" vm="112">
         <v>#VALUE!</v>
       </c>
       <c r="D122" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B123" t="s">
-        <v>161</v>
-      </c>
-      <c r="C123" t="e" vm="113">
-        <v>#VALUE!</v>
-      </c>
-      <c r="D123" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -5254,16 +5216,16 @@
     <hyperlink ref="D20" r:id="rId8" xr:uid="{5D1E9A79-DAED-4E54-94A0-2E050C0FB4FB}"/>
     <hyperlink ref="D21" r:id="rId9" xr:uid="{C1C49285-8EBC-473E-8C12-DBB157F3A8C2}"/>
     <hyperlink ref="D19" r:id="rId10" xr:uid="{1FF8D3EF-DD86-4DC1-830F-36FA2B59E905}"/>
-    <hyperlink ref="D35" r:id="rId11" xr:uid="{3F18330B-6975-4355-8A46-6C580C847FB3}"/>
-    <hyperlink ref="D36" r:id="rId12" xr:uid="{C6148396-714B-4295-8D91-B8D3001C92CA}"/>
-    <hyperlink ref="D37" r:id="rId13" xr:uid="{842AF9D9-E809-49FE-9404-90A2B38902D0}"/>
-    <hyperlink ref="D44" r:id="rId14" xr:uid="{98C4ACFA-B707-4EE2-A203-12CCB94EA8AB}"/>
-    <hyperlink ref="D45" r:id="rId15" xr:uid="{FAEE793E-398A-43F7-A7E8-E21E50AAA89C}"/>
-    <hyperlink ref="D46" r:id="rId16" xr:uid="{DDD7FAFB-B52A-4910-B6C6-F952981F5DE9}"/>
+    <hyperlink ref="D34" r:id="rId11" xr:uid="{3F18330B-6975-4355-8A46-6C580C847FB3}"/>
+    <hyperlink ref="D35" r:id="rId12" xr:uid="{C6148396-714B-4295-8D91-B8D3001C92CA}"/>
+    <hyperlink ref="D36" r:id="rId13" xr:uid="{842AF9D9-E809-49FE-9404-90A2B38902D0}"/>
+    <hyperlink ref="D43" r:id="rId14" xr:uid="{98C4ACFA-B707-4EE2-A203-12CCB94EA8AB}"/>
+    <hyperlink ref="D44" r:id="rId15" xr:uid="{FAEE793E-398A-43F7-A7E8-E21E50AAA89C}"/>
+    <hyperlink ref="D45" r:id="rId16" xr:uid="{DDD7FAFB-B52A-4910-B6C6-F952981F5DE9}"/>
     <hyperlink ref="D6" r:id="rId17" xr:uid="{71C7B438-B979-4DD3-B41E-8410DC6BB40F}"/>
-    <hyperlink ref="D99" r:id="rId18" xr:uid="{7973F455-F87D-4C0E-8E6D-35DA4F036127}"/>
-    <hyperlink ref="D94" r:id="rId19" xr:uid="{39576325-1274-4FA7-9777-858EDE57C1DA}"/>
-    <hyperlink ref="D96" r:id="rId20" xr:uid="{33ADE732-0962-4018-BC5A-6F2939A34058}"/>
+    <hyperlink ref="D98" r:id="rId18" xr:uid="{7973F455-F87D-4C0E-8E6D-35DA4F036127}"/>
+    <hyperlink ref="D93" r:id="rId19" xr:uid="{39576325-1274-4FA7-9777-858EDE57C1DA}"/>
+    <hyperlink ref="D95" r:id="rId20" xr:uid="{33ADE732-0962-4018-BC5A-6F2939A34058}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId21"/>

</xml_diff>